<commit_message>
update demo models 20260519
</commit_message>
<xml_diff>
--- a/models/demo-dk/demo-dk.xlsx
+++ b/models/demo-dk/demo-dk.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/shxie/Projects/anse-models/demo-dk/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/shxie/projects/anse-models/demo-dk/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1BE8870-300B-FD4D-8108-778F9FF2C026}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E52F5B9-A3E0-E146-9ABF-18B9BF595EF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22680" yWindow="2320" windowWidth="28520" windowHeight="23120" xr2:uid="{73351A0E-E394-C94F-8AB9-3EA9DA143F24}"/>
   </bookViews>
@@ -19,7 +19,7 @@
     <sheet name="Inputs - Spatial" sheetId="4" r:id="rId4"/>
     <sheet name="Inputs - Curves" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -44,6 +44,7 @@
   <authors>
     <author>Magnan, Michael</author>
     <author>mhafer</author>
+    <author>tc={6B69D804-0597-AE41-AD60-4FE944E7449C}</author>
   </authors>
   <commentList>
     <comment ref="D1" authorId="0" shapeId="0" xr:uid="{DE5AEED7-5306-0F41-A9F6-E09723C07087}">
@@ -380,27 +381,13 @@
         </r>
       </text>
     </comment>
-    <comment ref="G102" authorId="0" shapeId="0" xr:uid="{9D0C205B-9C9C-3F4A-912F-B707A4FF980A}">
+    <comment ref="G102" authorId="2" shapeId="0" xr:uid="{6B69D804-0597-AE41-AD60-4FE944E7449C}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color rgb="FF000000"/>
-            <rFont val="Helvetica Neue"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Magnan, Michael:
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    The physical state into which the C mass is transformed. Must supply a distinct Physical State here (not Physical State Group)
 </t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color rgb="FF000000"/>
-            <rFont val="Helvetica Neue"/>
-            <family val="2"/>
-          </rPr>
-          <t>The physical state into which the C mass is transformed. Must supply a distinct Physical State here (not Physical State Group)</t>
-        </r>
       </text>
     </comment>
   </commentList>
@@ -764,18 +751,9 @@
     <t>Proportion</t>
   </si>
   <si>
-    <t>Target Amount (Double precison)</t>
-  </si>
-  <si>
     <t>New Physical State Name</t>
   </si>
   <si>
-    <t>Filter By Physical State Name/Group</t>
-  </si>
-  <si>
-    <t>Filter By Species Name/Group</t>
-  </si>
-  <si>
     <t>Note</t>
   </si>
   <si>
@@ -1074,13 +1052,22 @@
   </si>
   <si>
     <t>Pulp and paper manufacturing Parameters, DK</t>
+  </si>
+  <si>
+    <t>Target</t>
+  </si>
+  <si>
+    <t>Physical State Rule</t>
+  </si>
+  <si>
+    <t>Species Rule</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1110,8 +1097,14 @@
       <color theme="1"/>
       <name val="HelveticaNeue"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1122,6 +1115,12 @@
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.14999847407452621"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="65"/>
       </patternFill>
     </fill>
   </fills>
@@ -1137,12 +1136,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1158,6 +1158,12 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Magnan, Michael" id="{AA844FE2-EB73-1C46-8CBC-258D2F726562}" userId="" providerId=""/>
+</personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1475,6 +1481,15 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="G102" personId="{AA844FE2-EB73-1C46-8CBC-258D2F726562}" id="{6B69D804-0597-AE41-AD60-4FE944E7449C}">
+    <text xml:space="preserve">The physical state into which the C mass is transformed. Must supply a distinct Physical State here (not Physical State Group)
+</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F935C300-5F44-C54A-ADD4-2A504DCCAD49}">
   <dimension ref="B1:L129"/>
@@ -1534,7 +1549,7 @@
         <v>11</v>
       </c>
       <c r="C3" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="D3">
         <f>'Inputs - Spatial'!$C$2</f>
@@ -1549,7 +1564,7 @@
         <v>11</v>
       </c>
       <c r="C4" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="D4">
         <f>'Inputs - Spatial'!$C$2</f>
@@ -1564,7 +1579,7 @@
         <v>11</v>
       </c>
       <c r="C5" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="D5">
         <f>'Inputs - Spatial'!$C$2</f>
@@ -1579,7 +1594,7 @@
         <v>11</v>
       </c>
       <c r="C7" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="D7">
         <f>'Inputs - Spatial'!$C$2</f>
@@ -1591,7 +1606,7 @@
         <v>11</v>
       </c>
       <c r="C8" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="D8">
         <f>'Inputs - Spatial'!$C$2</f>
@@ -1603,14 +1618,14 @@
         <v>11</v>
       </c>
       <c r="C9" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="D9">
         <f>'Inputs - Spatial'!$C$2</f>
         <v>45</v>
       </c>
       <c r="E9" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="11" spans="2:12" ht="16" customHeight="1">
@@ -1618,7 +1633,7 @@
         <v>11</v>
       </c>
       <c r="C11" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="D11">
         <f>'Inputs - Spatial'!$C$2</f>
@@ -1630,7 +1645,7 @@
         <v>11</v>
       </c>
       <c r="C12" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="D12">
         <f>'Inputs - Spatial'!$C$2</f>
@@ -1642,14 +1657,14 @@
         <v>11</v>
       </c>
       <c r="C13" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="D13">
         <f>'Inputs - Spatial'!$C$2</f>
         <v>45</v>
       </c>
       <c r="E13" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="15" spans="2:12" ht="16" customHeight="1">
@@ -1657,7 +1672,7 @@
         <v>11</v>
       </c>
       <c r="C15" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="D15">
         <f>'Inputs - Spatial'!$C$2</f>
@@ -1669,7 +1684,7 @@
         <v>11</v>
       </c>
       <c r="C17" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="D17">
         <f>'Inputs - Spatial'!$C$2</f>
@@ -1681,14 +1696,14 @@
         <v>11</v>
       </c>
       <c r="C18" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="D18">
         <f>'Inputs - Spatial'!$C$2</f>
         <v>45</v>
       </c>
       <c r="E18" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20" spans="2:12" ht="16" customHeight="1">
@@ -1696,7 +1711,7 @@
         <v>11</v>
       </c>
       <c r="C20" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="D20">
         <f>'Inputs - Spatial'!$C$2</f>
@@ -1708,7 +1723,7 @@
         <v>11</v>
       </c>
       <c r="C22" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="D22">
         <f>'Inputs - Spatial'!$C$2</f>
@@ -1720,7 +1735,7 @@
         <v>11</v>
       </c>
       <c r="C23" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="D23">
         <f>'Inputs - Spatial'!$C$2</f>
@@ -1732,7 +1747,7 @@
         <v>11</v>
       </c>
       <c r="C24" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="D24">
         <f>'Inputs - Spatial'!$C$2</f>
@@ -1779,7 +1794,7 @@
         <v>20</v>
       </c>
       <c r="C28" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="D28" t="str">
         <f>C40</f>
@@ -1795,7 +1810,7 @@
         <v>20</v>
       </c>
       <c r="C29" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="D29" t="str">
         <f t="shared" ref="D29:D36" si="0">C41</f>
@@ -1811,7 +1826,7 @@
         <v>20</v>
       </c>
       <c r="C30" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="D30" t="str">
         <f t="shared" si="0"/>
@@ -1827,7 +1842,7 @@
         <v>20</v>
       </c>
       <c r="C31" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="D31" t="str">
         <f t="shared" si="0"/>
@@ -1860,7 +1875,7 @@
         <v>20</v>
       </c>
       <c r="C33" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D33" t="str">
         <f t="shared" si="0"/>
@@ -1876,7 +1891,7 @@
         <v>20</v>
       </c>
       <c r="C34" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="D34" t="str">
         <f t="shared" si="0"/>
@@ -1892,7 +1907,7 @@
         <v>20</v>
       </c>
       <c r="C35" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="D35" t="str">
         <f t="shared" si="0"/>
@@ -1908,7 +1923,7 @@
         <v>20</v>
       </c>
       <c r="C36" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="D36" t="str">
         <f t="shared" si="0"/>
@@ -1929,74 +1944,74 @@
     </row>
     <row r="40" spans="2:5" ht="16" customHeight="1">
       <c r="B40" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="C40" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
     </row>
     <row r="41" spans="2:5" ht="16" customHeight="1">
       <c r="B41" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="C41" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="42" spans="2:5" ht="16" customHeight="1">
       <c r="B42" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="C42" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="43" spans="2:5" ht="16" customHeight="1">
       <c r="B43" t="s">
+        <v>121</v>
+      </c>
+      <c r="C43" t="s">
         <v>124</v>
-      </c>
-      <c r="C43" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="44" spans="2:5" ht="16" customHeight="1">
       <c r="B44" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="C44" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="45" spans="2:5" ht="16" customHeight="1">
       <c r="B45" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="C45" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
     </row>
     <row r="46" spans="2:5" ht="16" customHeight="1">
       <c r="B46" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="C46" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="47" spans="2:5" ht="16" customHeight="1">
       <c r="B47" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="C47" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="48" spans="2:5" ht="16" customHeight="1">
       <c r="B48" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="C48" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
     </row>
     <row r="50" spans="2:7" s="3" customFormat="1" ht="16" customHeight="1">
@@ -2598,7 +2613,7 @@
         <v>35</v>
       </c>
       <c r="C92" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="D92" t="str">
         <f>C40</f>
@@ -2614,7 +2629,7 @@
         <v>35</v>
       </c>
       <c r="C93" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="D93" t="str">
         <f t="shared" ref="D93:D95" si="1">C41</f>
@@ -2630,7 +2645,7 @@
         <v>35</v>
       </c>
       <c r="C94" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="D94" t="str">
         <f t="shared" si="1"/>
@@ -2646,7 +2661,7 @@
         <v>35</v>
       </c>
       <c r="C95" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="D95" t="str">
         <f t="shared" si="1"/>
@@ -2662,7 +2677,7 @@
         <v>35</v>
       </c>
       <c r="C96" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="D96" t="str">
         <f>C44</f>
@@ -2678,7 +2693,7 @@
         <v>35</v>
       </c>
       <c r="C97" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D97" t="str">
         <f>C45</f>
@@ -2694,7 +2709,7 @@
         <v>35</v>
       </c>
       <c r="C98" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="D98" t="str">
         <f>C46</f>
@@ -2710,7 +2725,7 @@
         <v>35</v>
       </c>
       <c r="C99" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="D99" t="str">
         <f>C47</f>
@@ -2726,7 +2741,7 @@
         <v>35</v>
       </c>
       <c r="C100" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="D100" t="str">
         <f>C48</f>
@@ -2750,25 +2765,25 @@
       <c r="E102" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="F102" s="3" t="s">
+      <c r="F102" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="G102" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="G102" s="3" t="s">
+      <c r="H102" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="I102" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="J102" s="3" t="s">
         <v>40</v>
-      </c>
-      <c r="H102" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="I102" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="J102" s="3" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="104" spans="2:10" ht="16" customHeight="1">
       <c r="B104" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C104" t="str" cm="1">
         <f t="array" ref="C104">C92</f>
@@ -2783,7 +2798,7 @@
     </row>
     <row r="105" spans="2:10" ht="16" customHeight="1">
       <c r="B105" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C105" t="str" cm="1">
         <f t="array" ref="C105">C92</f>
@@ -2798,7 +2813,7 @@
     </row>
     <row r="107" spans="2:10" ht="16" customHeight="1">
       <c r="B107" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C107" t="str" cm="1">
         <f t="array" ref="C107">C93</f>
@@ -2813,7 +2828,7 @@
     </row>
     <row r="108" spans="2:10" ht="16" customHeight="1">
       <c r="B108" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C108" t="str" cm="1">
         <f t="array" ref="C108">C93</f>
@@ -2828,7 +2843,7 @@
     </row>
     <row r="110" spans="2:10" ht="16" customHeight="1">
       <c r="B110" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C110" t="str" cm="1">
         <f t="array" ref="C110">C94</f>
@@ -2843,7 +2858,7 @@
     </row>
     <row r="111" spans="2:10" ht="16" customHeight="1">
       <c r="B111" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C111" t="str" cm="1">
         <f t="array" ref="C111">C94</f>
@@ -2858,7 +2873,7 @@
     </row>
     <row r="113" spans="2:5" ht="16" customHeight="1">
       <c r="B113" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C113" t="str" cm="1">
         <f t="array" ref="C113">C95</f>
@@ -2873,7 +2888,7 @@
     </row>
     <row r="114" spans="2:5" ht="16" customHeight="1">
       <c r="B114" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C114" t="str" cm="1">
         <f t="array" ref="C114">C95</f>
@@ -2888,7 +2903,7 @@
     </row>
     <row r="116" spans="2:5" ht="16" customHeight="1">
       <c r="B116" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C116" t="str">
         <f>C96</f>
@@ -2903,7 +2918,7 @@
     </row>
     <row r="118" spans="2:5" ht="16" customHeight="1">
       <c r="B118" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C118" t="str" cm="1">
         <f t="array" ref="C118">C97</f>
@@ -2918,7 +2933,7 @@
     </row>
     <row r="119" spans="2:5" ht="16" customHeight="1">
       <c r="B119" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C119" t="str" cm="1">
         <f t="array" ref="C119">C97</f>
@@ -2933,7 +2948,7 @@
     </row>
     <row r="121" spans="2:5" ht="16" customHeight="1">
       <c r="B121" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C121" t="str" cm="1">
         <f t="array" ref="C121">C98</f>
@@ -2948,7 +2963,7 @@
     </row>
     <row r="122" spans="2:5" ht="16" customHeight="1">
       <c r="B122" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C122" t="str" cm="1">
         <f t="array" ref="C122">C98</f>
@@ -2963,7 +2978,7 @@
     </row>
     <row r="124" spans="2:5" ht="16" customHeight="1">
       <c r="B124" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C124" t="str" cm="1">
         <f t="array" ref="C124">C99</f>
@@ -2978,7 +2993,7 @@
     </row>
     <row r="125" spans="2:5" ht="16" customHeight="1">
       <c r="B125" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C125" t="str" cm="1">
         <f t="array" ref="C125">C99</f>
@@ -2993,7 +3008,7 @@
     </row>
     <row r="127" spans="2:5" ht="16" customHeight="1">
       <c r="B127" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C127" t="str" cm="1">
         <f t="array" ref="C127">C100</f>
@@ -3008,7 +3023,7 @@
     </row>
     <row r="128" spans="2:5" ht="16" customHeight="1">
       <c r="B128" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C128" t="str" cm="1">
         <f t="array" ref="C128">C100</f>
@@ -3023,7 +3038,7 @@
     </row>
     <row r="129" spans="2:5" ht="16" customHeight="1">
       <c r="B129" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C129" t="str" cm="1">
         <f t="array" ref="C129">C100</f>
@@ -3060,31 +3075,31 @@
   <sheetData>
     <row r="1" spans="2:11" s="3" customFormat="1">
       <c r="B1" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="G1" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="H1" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>51</v>
-      </c>
       <c r="I1" s="3" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="K1" s="3" t="s">
         <v>34</v>
@@ -3092,7 +3107,7 @@
     </row>
     <row r="3" spans="2:11">
       <c r="B3" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C3" t="str">
         <f>'Inputs - Flow Network'!C3</f>
@@ -3131,26 +3146,26 @@
   <sheetData>
     <row r="1" spans="2:7" s="3" customFormat="1">
       <c r="B1" s="2" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" spans="2:7">
       <c r="B3" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C3" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5" spans="2:7" s="3" customFormat="1">
       <c r="B5" s="2" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>1</v>
@@ -3164,27 +3179,27 @@
     </row>
     <row r="7" spans="2:7" s="3" customFormat="1">
       <c r="B7" s="2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
     </row>
     <row r="9" spans="2:7" s="3" customFormat="1">
       <c r="B9" s="2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>1</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="F9" s="3" t="s">
         <v>33</v>
@@ -3195,7 +3210,7 @@
     </row>
     <row r="11" spans="2:7" s="3" customFormat="1">
       <c r="B11" s="2" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>1</v>
@@ -3209,24 +3224,24 @@
     </row>
     <row r="13" spans="2:7" s="3" customFormat="1">
       <c r="B13" s="2" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="15" spans="2:7" s="3" customFormat="1">
       <c r="B15" s="2" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>1</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>34</v>
@@ -3255,22 +3270,22 @@
   <sheetData>
     <row r="1" spans="2:8" s="3" customFormat="1">
       <c r="B1" s="2" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>1</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>34</v>
@@ -3278,13 +3293,13 @@
     </row>
     <row r="2" spans="2:8">
       <c r="B2" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C2">
         <v>45</v>
       </c>
       <c r="D2" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -3292,7 +3307,7 @@
     </row>
     <row r="5" spans="2:8" s="3" customFormat="1">
       <c r="B5" s="2" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>1</v>
@@ -3300,21 +3315,21 @@
     </row>
     <row r="6" spans="2:8">
       <c r="B6" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="C6" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="8" spans="2:8" s="3" customFormat="1">
       <c r="B8" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>1</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>34</v>
@@ -3322,10 +3337,10 @@
     </row>
     <row r="10" spans="2:8">
       <c r="B10" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C10" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="D10" t="str">
         <f>C6</f>
@@ -3334,21 +3349,21 @@
     </row>
     <row r="12" spans="2:8" s="3" customFormat="1">
       <c r="B12" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>19</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
     </row>
     <row r="13" spans="2:8">
       <c r="B13" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C13" t="str">
         <f>C10</f>
@@ -3379,13 +3394,13 @@
   <sheetData>
     <row r="1" spans="2:6" s="3" customFormat="1">
       <c r="B1" s="2" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>33</v>
@@ -3396,7 +3411,7 @@
     </row>
     <row r="3" spans="2:6" s="3" customFormat="1">
       <c r="B3" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>1</v>
@@ -3410,33 +3425,33 @@
     </row>
     <row r="5" spans="2:6" s="3" customFormat="1">
       <c r="B5" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>19</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
     </row>
     <row r="7" spans="2:6" s="3" customFormat="1">
       <c r="B7" s="2" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C7" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>96</v>
-      </c>
       <c r="E7" s="2" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
   </sheetData>

</xml_diff>